<commit_message>
stabilize vercel + codespace connection
</commit_message>
<xml_diff>
--- a/data/master update.xlsx
+++ b/data/master update.xlsx
@@ -1,15 +1,15 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="680" yWindow="760" windowWidth="28040" windowHeight="17200" tabRatio="600" firstSheet="0" activeTab="1" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="download" sheetId="1" state="visible" r:id="rId1"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="screening" sheetId="2" state="visible" r:id="rId2"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="turnitin" sheetId="3" state="visible" r:id="rId3"/>
-    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="upload" sheetId="4" state="visible" r:id="rId4"/>
+    <sheet name="download" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet name="screening" sheetId="2" state="visible" r:id="rId2"/>
+    <sheet name="turnitin" sheetId="3" state="visible" r:id="rId3"/>
+    <sheet name="upload" sheetId="4" state="visible" r:id="rId4"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1"/>
@@ -563,7 +563,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:E18"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="25"/>
   <cols>
     <col width="22" customWidth="1" style="1" min="1" max="1"/>
     <col width="18" customWidth="1" style="1" min="2" max="2"/>
@@ -1071,7 +1071,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Y17"/>
+  <dimension ref="A1:Y18"/>
   <sheetFormatPr baseColWidth="10" defaultRowHeight="16"/>
   <sheetData>
     <row r="1">
@@ -3198,6 +3198,48 @@
       <c r="Y17" t="inlineStr">
         <is>
           <t>/Users/nasruddinmadon/turnitin-assistant-v5.7.1/storage/template_screening_reports/needs_review</t>
+        </is>
+      </c>
+    </row>
+    <row r="18">
+      <c r="A18" t="inlineStr">
+        <is>
+          <t>2026-05-21 10:12:34</t>
+        </is>
+      </c>
+      <c r="B18" t="inlineStr">
+        <is>
+          <t>26815</t>
+        </is>
+      </c>
+      <c r="C18" t="inlineStr">
+        <is>
+          <t>MAT RIPIN et al.</t>
+        </is>
+      </c>
+      <c r="D18" t="inlineStr">
+        <is>
+          <t>LUBRICATION STRATEGIES IN MAGNESIUM ALLOY MACHINING: A SYSTEMATIC REVIEW FROM DRY MACHINING TO VEGETABLE OIL-BASED NANO-MQL</t>
+        </is>
+      </c>
+      <c r="E18" t="inlineStr">
+        <is>
+          <t>storage/ojs-downloads/26815/SLR_Lubrication Strategies Magnesium Alloy Machining.doc</t>
+        </is>
+      </c>
+      <c r="F18" t="inlineStr">
+        <is>
+          <t>SCREENING ERROR</t>
+        </is>
+      </c>
+      <c r="L18" t="inlineStr">
+        <is>
+          <t>DOCX to PDF conversion failed.</t>
+        </is>
+      </c>
+      <c r="M18" t="inlineStr">
+        <is>
+          <t>2026-05-21 03:39:05</t>
         </is>
       </c>
     </row>
@@ -3213,7 +3255,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="25"/>
   <cols>
     <col width="26.83203125" customWidth="1" style="13" min="1" max="1"/>
     <col width="40.33203125" customWidth="1" style="13" min="2" max="2"/>
@@ -3266,7 +3308,7 @@
     <pageSetUpPr/>
   </sheetPr>
   <dimension ref="A1:F1"/>
-  <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="25" outlineLevelCol="0"/>
+  <sheetFormatPr baseColWidth="10" defaultColWidth="50.83203125" defaultRowHeight="25"/>
   <cols>
     <col width="26.83203125" customWidth="1" style="5" min="1" max="1"/>
     <col width="40.33203125" customWidth="1" style="5" min="2" max="2"/>

</xml_diff>